<commit_message>
client intake: lecturer availability is entered as unavailable slots directly (no complement) and the shared-course example uses the real Electrical & Electronic Engineering name
</commit_message>
<xml_diff>
--- a/docs/client_intake/courses_template.xlsx
+++ b/docs/client_intake/courses_template.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Computer Engineering | Electrical Engineering</t>
+          <t>Computer Engineering | Electrical &amp; Electronic Engineering</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -597,7 +597,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Department name in this faculty. To share ONE course across departments, list them separated by | (first owns it), e.g. Computer Engineering | Electrical Engineering.</t>
+          <t>Department name in this faculty. To share ONE course across departments, list them separated by | (first owns it), e.g. Computer Engineering | Electrical &amp; Electronic Engineering.</t>
         </is>
       </c>
     </row>

</xml_diff>